<commit_message>
Add cost details sheet to resource tracker
March 2026 AWS cost breakdown by service, daily spend trend,
monthly projection (~$1,100/mo with GST), and 8 optimization
recommendations with potential 46% cost reduction ($504/mo savings).
Top item: upgrade EKS from v1.31 extended support to save $365/mo.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LinkedEye_AWS_Resource_Tracker.xlsx
+++ b/LinkedEye_AWS_Resource_Tracker.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Tools &amp; Services" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Deleted Resources" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Credentials &amp; Access" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Cost Details" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,8 +21,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="4">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+  </numFmts>
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,8 +44,12 @@
     <font>
       <color rgb="00CC0000"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -77,6 +84,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFC7CE"/>
         <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -126,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -149,6 +162,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4587,11 +4613,11 @@
           <t>TOOL CREDENTIALS</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
+      <c r="B2" s="8" t="n"/>
+      <c r="C2" s="8" t="n"/>
+      <c r="D2" s="8" t="n"/>
+      <c r="E2" s="8" t="n"/>
+      <c r="F2" s="9" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -4792,11 +4818,11 @@
           <t>VAULT UNSEAL KEYS (need 3 of 5 to unseal)</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
+      <c r="B9" s="8" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -4972,11 +4998,11 @@
           <t>POSTGRESQL DATABASE CREDENTIALS</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="n"/>
+      <c r="F16" s="9" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -5212,11 +5238,11 @@
           <t>SSH ACCESS</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="8" t="n"/>
+      <c r="F25" s="9" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -5320,11 +5346,11 @@
           <t>AWS ACCOUNT ACCESS</t>
         </is>
       </c>
-      <c r="B29" s="3" t="n"/>
-      <c r="C29" s="3" t="n"/>
-      <c r="D29" s="3" t="n"/>
-      <c r="E29" s="3" t="n"/>
-      <c r="F29" s="3" t="n"/>
+      <c r="B29" s="8" t="n"/>
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="8" t="n"/>
+      <c r="E29" s="8" t="n"/>
+      <c r="F29" s="9" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -5396,11 +5422,11 @@
           <t>ALB ENDPOINTS (linkedeye-tools-alb)</t>
         </is>
       </c>
-      <c r="B32" s="3" t="n"/>
-      <c r="C32" s="3" t="n"/>
-      <c r="D32" s="3" t="n"/>
-      <c r="E32" s="3" t="n"/>
-      <c r="F32" s="3" t="n"/>
+      <c r="B32" s="8" t="n"/>
+      <c r="C32" s="8" t="n"/>
+      <c r="D32" s="8" t="n"/>
+      <c r="E32" s="8" t="n"/>
+      <c r="F32" s="9" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -5504,11 +5530,11 @@
           <t>VAULT UNSEAL PROCEDURE (after restart)</t>
         </is>
       </c>
-      <c r="B36" s="3" t="n"/>
-      <c r="C36" s="3" t="n"/>
-      <c r="D36" s="3" t="n"/>
-      <c r="E36" s="3" t="n"/>
-      <c r="F36" s="3" t="n"/>
+      <c r="B36" s="8" t="n"/>
+      <c r="C36" s="8" t="n"/>
+      <c r="D36" s="8" t="n"/>
+      <c r="E36" s="8" t="n"/>
+      <c r="F36" s="9" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -5668,11 +5694,11 @@
           <t>DATABASE BACKUP</t>
         </is>
       </c>
-      <c r="B42" s="3" t="n"/>
-      <c r="C42" s="3" t="n"/>
-      <c r="D42" s="3" t="n"/>
-      <c r="E42" s="3" t="n"/>
-      <c r="F42" s="3" t="n"/>
+      <c r="B42" s="8" t="n"/>
+      <c r="C42" s="8" t="n"/>
+      <c r="D42" s="8" t="n"/>
+      <c r="E42" s="8" t="n"/>
+      <c r="F42" s="9" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -5719,4 +5745,1703 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F83"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>LinkedEye AWS Cost Report — March 2026 (Estimated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>AWS Service</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>March 2026 (USD)</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>% of Total</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Resource</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Usage</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Optimization Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Amazon EC2 — Compute</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="n">
+        <v>322.93</v>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>37.0%</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>2x m5.xlarge (node groups) + m5.2xlarge + m5.4xlarge</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>853h m5.xlarge, 174h m5.2xlarge, 97h m5.4xlarge</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>m5.4xlarge terminated mid-month; consider Reserved Instances for steady-state nodes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Amazon EKS — Control Plane</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="n">
+        <v>44.65</v>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>5.1%</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>linkedeye-finspot-k8s-cluster</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>446 cluster-hours</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Fixed $0.10/hr — no optimization possible</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Amazon EKS — Extended Support</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>223.26</v>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>25.6%</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>EKS v1.31 extended support surcharge</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>446 hours @ $0.50/hr</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>UPGRADE to v1.32+ when available to exit extended support ($0.50/hr savings)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Amazon EKS — Hybrid Nodes</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="n">
+        <v>53.05</v>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>6.1%</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>On-prem hybrid node vCPU hours</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>2,652 vCPU-hours</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Scales with client count; currently 15 clients</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>EC2 Other (EBS)</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="n">
+        <v>35.66</v>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>4.1%</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>gp3: 322GB, gp2: 54GB</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>50GB + 100GB node disks + snapshots</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Migrate gp2 → gp3 for cost savings</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Elastic Load Balancing</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>12.93</v>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>1.5%</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>linkedeye-tools-alb</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>541 ALB-hours</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Fixed cost — single ALB is efficient</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Amazon VPC (Public IPv4)</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="n">
+        <v>12.75</v>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>1.5%</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>2 ALB EIPs + node public IPs</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>2,549 IP-hours</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Release unused EIPs if any</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Amazon VPC (NAT Gateway)</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="n">
+        <v>18.76</v>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>2.2%</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>NAT Gateway hours</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>335 hours</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>NAT GW not in state table — verify if still needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Amazon CloudWatch</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="n">
+        <v>10.33</v>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>1.2%</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>VPC Flow Logs, EKS logs</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>20.4 GB vended logs</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Set retention on EKS logs (currently unlimited — 2.98 GB growing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>AWS WAF</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="n">
+        <v>5.35</v>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>0.6%</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>linkedeye-waf (4 rules)</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>1 WebACL + 4 rules</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Standard pricing — already minimal</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>AWS KMS</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>0.1%</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>3 keys (EKS, Vault, EBS)</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>3 active keys</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Delete orphaned key d514cb7e to save $1/mo</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Amazon S3</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Velero + Audit log buckets</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Minimal storage</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>AWS CloudTrail</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Audit logging</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Free tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Amazon GuardDuty</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Threat detection</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Free tier / trial</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Amazon EFS</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>fs-50094f81 (finspot-cloud VPC)</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Minimal</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Orphaned — delete when possible</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Tax (GST 18%)</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="n">
+        <v>133.34</v>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>15.3%</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>India GST on AWS services</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>TOTAL (March 2026 estimated)</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="n">
+        <v>873.75</v>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr"/>
+      <c r="E20" s="13" t="inlineStr"/>
+      <c r="F20" s="13" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>DAILY SPEND TREND — March 2026</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n"/>
+      <c r="C22" s="3" t="n"/>
+      <c r="D22" s="3" t="n"/>
+      <c r="E22" s="3" t="n"/>
+      <c r="F22" s="3" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>Daily Cost (USD)</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>Cumulative (USD)</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr"/>
+      <c r="F23" s="15" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="n">
+        <v>133.34</v>
+      </c>
+      <c r="C24" s="12" t="n">
+        <v>133.34</v>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Tax payment</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr"/>
+      <c r="F24" s="4" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="12" t="n">
+        <v>133.34</v>
+      </c>
+      <c r="D25" s="4" t="inlineStr"/>
+      <c r="E25" s="4" t="inlineStr"/>
+      <c r="F25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="12" t="n">
+        <v>133.34</v>
+      </c>
+      <c r="D26" s="4" t="inlineStr"/>
+      <c r="E26" s="4" t="inlineStr"/>
+      <c r="F26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="12" t="n">
+        <v>133.34</v>
+      </c>
+      <c r="D27" s="4" t="inlineStr"/>
+      <c r="E27" s="4" t="inlineStr"/>
+      <c r="F27" s="4" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="12" t="n">
+        <v>133.34</v>
+      </c>
+      <c r="D28" s="4" t="inlineStr"/>
+      <c r="E28" s="4" t="inlineStr"/>
+      <c r="F28" s="4" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C29" s="12" t="n">
+        <v>133.94</v>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Initial setup begins</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr"/>
+      <c r="F29" s="4" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="n">
+        <v>26.75</v>
+      </c>
+      <c r="C30" s="12" t="n">
+        <v>160.69</v>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>VPC + subnets created</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr"/>
+      <c r="F30" s="4" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="n">
+        <v>33.37</v>
+      </c>
+      <c r="C31" s="12" t="n">
+        <v>194.06</v>
+      </c>
+      <c r="D31" s="4" t="inlineStr"/>
+      <c r="E31" s="4" t="inlineStr"/>
+      <c r="F31" s="4" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="n">
+        <v>33.37</v>
+      </c>
+      <c r="C32" s="12" t="n">
+        <v>227.43</v>
+      </c>
+      <c r="D32" s="4" t="inlineStr"/>
+      <c r="E32" s="4" t="inlineStr"/>
+      <c r="F32" s="4" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="n">
+        <v>50.82</v>
+      </c>
+      <c r="C33" s="12" t="n">
+        <v>278.25</v>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>EKS cluster + enterprise setup</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr"/>
+      <c r="F33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="n">
+        <v>32.21</v>
+      </c>
+      <c r="C34" s="12" t="n">
+        <v>310.46</v>
+      </c>
+      <c r="D34" s="4" t="inlineStr"/>
+      <c r="E34" s="4" t="inlineStr"/>
+      <c r="F34" s="4" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="n">
+        <v>24.46</v>
+      </c>
+      <c r="C35" s="12" t="n">
+        <v>334.92</v>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>EKS addons + ALB + KMS</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr"/>
+      <c r="F35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="n">
+        <v>28.71</v>
+      </c>
+      <c r="C36" s="12" t="n">
+        <v>363.6299999999999</v>
+      </c>
+      <c r="D36" s="4" t="inlineStr"/>
+      <c r="E36" s="4" t="inlineStr"/>
+      <c r="F36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="B37" s="12" t="n">
+        <v>28.71</v>
+      </c>
+      <c r="C37" s="12" t="n">
+        <v>392.3399999999999</v>
+      </c>
+      <c r="D37" s="4" t="inlineStr"/>
+      <c r="E37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="n">
+        <v>29.65</v>
+      </c>
+      <c r="C38" s="12" t="n">
+        <v>421.9899999999999</v>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Hybrid node role created</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr"/>
+      <c r="F38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="C39" s="12" t="n">
+        <v>454.4899999999999</v>
+      </c>
+      <c r="D39" s="4" t="inlineStr"/>
+      <c r="E39" s="4" t="inlineStr"/>
+      <c r="F39" s="4" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="n">
+        <v>36.57</v>
+      </c>
+      <c r="C40" s="12" t="n">
+        <v>491.0599999999999</v>
+      </c>
+      <c r="D40" s="4" t="inlineStr"/>
+      <c r="E40" s="4" t="inlineStr"/>
+      <c r="F40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="n">
+        <v>43.28</v>
+      </c>
+      <c r="C41" s="12" t="n">
+        <v>534.3399999999999</v>
+      </c>
+      <c r="D41" s="4" t="inlineStr"/>
+      <c r="E41" s="4" t="inlineStr"/>
+      <c r="F41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="n">
+        <v>41.29</v>
+      </c>
+      <c r="C42" s="12" t="n">
+        <v>575.6299999999999</v>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Node groups launched (peak day)</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr"/>
+      <c r="F42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="n">
+        <v>32.26</v>
+      </c>
+      <c r="C43" s="12" t="n">
+        <v>607.8899999999999</v>
+      </c>
+      <c r="D43" s="4" t="inlineStr"/>
+      <c r="E43" s="4" t="inlineStr"/>
+      <c r="F43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B44" s="12" t="n">
+        <v>31.09</v>
+      </c>
+      <c r="C44" s="12" t="n">
+        <v>638.9799999999999</v>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Steady state begins (~$31/day)</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr"/>
+      <c r="F44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="n">
+        <v>31.13</v>
+      </c>
+      <c r="C45" s="12" t="n">
+        <v>670.1099999999999</v>
+      </c>
+      <c r="D45" s="4" t="inlineStr"/>
+      <c r="E45" s="4" t="inlineStr"/>
+      <c r="F45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B46" s="12" t="n">
+        <v>31.09</v>
+      </c>
+      <c r="C46" s="12" t="n">
+        <v>701.1999999999999</v>
+      </c>
+      <c r="D46" s="4" t="inlineStr"/>
+      <c r="E46" s="4" t="inlineStr"/>
+      <c r="F46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B47" s="12" t="n">
+        <v>31.07</v>
+      </c>
+      <c r="C47" s="12" t="n">
+        <v>732.27</v>
+      </c>
+      <c r="D47" s="4" t="inlineStr"/>
+      <c r="E47" s="4" t="inlineStr"/>
+      <c r="F47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B48" s="12" t="n">
+        <v>31.07</v>
+      </c>
+      <c r="C48" s="12" t="n">
+        <v>763.34</v>
+      </c>
+      <c r="D48" s="4" t="inlineStr"/>
+      <c r="E48" s="4" t="inlineStr"/>
+      <c r="F48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B49" s="12" t="n">
+        <v>31.07</v>
+      </c>
+      <c r="C49" s="12" t="n">
+        <v>794.4100000000001</v>
+      </c>
+      <c r="D49" s="4" t="inlineStr"/>
+      <c r="E49" s="4" t="inlineStr"/>
+      <c r="F49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B50" s="12" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="C50" s="12" t="n">
+        <v>825.5100000000001</v>
+      </c>
+      <c r="D50" s="4" t="inlineStr"/>
+      <c r="E50" s="4" t="inlineStr"/>
+      <c r="F50" s="4" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B51" s="12" t="n">
+        <v>31.08</v>
+      </c>
+      <c r="C51" s="12" t="n">
+        <v>856.5900000000001</v>
+      </c>
+      <c r="D51" s="4" t="inlineStr"/>
+      <c r="E51" s="4" t="inlineStr"/>
+      <c r="F51" s="4" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B52" s="12" t="n">
+        <v>17.48</v>
+      </c>
+      <c r="C52" s="12" t="n">
+        <v>874.0700000000002</v>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>Partial day (billing in progress)</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr"/>
+      <c r="F52" s="4" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>MONTHLY COST PROJECTION</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n"/>
+      <c r="C54" s="3" t="n"/>
+      <c r="D54" s="3" t="n"/>
+      <c r="E54" s="3" t="n"/>
+      <c r="F54" s="3" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="15" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="B55" s="15" t="inlineStr">
+        <is>
+          <t>Estimated Cost (USD)</t>
+        </is>
+      </c>
+      <c r="C55" s="15" t="inlineStr">
+        <is>
+          <t>Breakdown</t>
+        </is>
+      </c>
+      <c r="D55" s="15" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="E55" s="15" t="inlineStr"/>
+      <c r="F55" s="15" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>March 2026 (actual)</t>
+        </is>
+      </c>
+      <c r="B56" s="12" t="n">
+        <v>874.08</v>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>29 days billed so far</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Estimated — final bill pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Steady-state daily run rate</t>
+        </is>
+      </c>
+      <c r="B57" s="12" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Per day from Mar 21-28 avg</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>After initial setup costs settled</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>Projected monthly (30 days)</t>
+        </is>
+      </c>
+      <c r="B58" s="12" t="n">
+        <v>933</v>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>$31.10/day x 30</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Excluding tax</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Projected monthly (with 18% GST)</t>
+        </is>
+      </c>
+      <c r="B59" s="12" t="n">
+        <v>1100.94</v>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>$933 + 18% tax</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Full monthly estimate</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr"/>
+      <c r="B60" s="4" t="inlineStr"/>
+      <c r="C60" s="4" t="inlineStr"/>
+      <c r="D60" s="4" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>COST BREAKDOWN (steady state/mo)</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr"/>
+      <c r="C61" s="4" t="inlineStr"/>
+      <c r="D61" s="4" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  EKS Control Plane</t>
+        </is>
+      </c>
+      <c r="B62" s="12" t="n">
+        <v>73</v>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>$0.10/hr x 730hr</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  EKS Extended Support</t>
+        </is>
+      </c>
+      <c r="B63" s="12" t="n">
+        <v>365</v>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>$0.50/hr x 730hr</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>LARGEST COST — upgrade EKS to exit</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  EC2 Nodes (2x m5.xlarge)</t>
+        </is>
+      </c>
+      <c r="B64" s="12" t="n">
+        <v>280</v>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>$0.192/hr x 2 x 730hr</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>Consider Reserved Instances (40% savings)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  EKS Hybrid Nodes</t>
+        </is>
+      </c>
+      <c r="B65" s="12" t="n">
+        <v>55</v>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>~15 clients, 2 vCPU each</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>Scales with clients</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  EBS Volumes</t>
+        </is>
+      </c>
+      <c r="B66" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>150GB gp3</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ALB</t>
+        </is>
+      </c>
+      <c r="B67" s="12" t="n">
+        <v>22</v>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>$0.03/hr + LCU</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CloudWatch Logs</t>
+        </is>
+      </c>
+      <c r="B68" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>~20GB/mo</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>Set retention to reduce</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  VPC (Public IPs)</t>
+        </is>
+      </c>
+      <c r="B69" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>~4 public IPv4</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  WAF</t>
+        </is>
+      </c>
+      <c r="B70" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>1 ACL + 4 rules</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Other (KMS, S3, etc.)</t>
+        </is>
+      </c>
+      <c r="B71" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>Minimal</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>COST OPTIMIZATION RECOMMENDATIONS</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="n"/>
+      <c r="C73" s="3" t="n"/>
+      <c r="D73" s="3" t="n"/>
+      <c r="E73" s="3" t="n"/>
+      <c r="F73" s="3" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="15" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B74" s="15" t="inlineStr">
+        <is>
+          <t>Recommendation</t>
+        </is>
+      </c>
+      <c r="C74" s="15" t="inlineStr">
+        <is>
+          <t>Estimated Savings/mo</t>
+        </is>
+      </c>
+      <c r="D74" s="15" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="E74" s="15" t="inlineStr">
+        <is>
+          <t>Effort</t>
+        </is>
+      </c>
+      <c r="F74" s="15" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>Upgrade EKS to v1.32+ (exit extended support)</t>
+        </is>
+      </c>
+      <c r="C75" s="12" t="n">
+        <v>365</v>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>EKS v1.31 extended support costs $0.50/hr ($365/mo). Upgrading removes this. Largest single savings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>Reserved Instances for m5.xlarge nodes</t>
+        </is>
+      </c>
+      <c r="C76" s="12" t="n">
+        <v>112</v>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>2x m5.xlarge at RI 1-year no-upfront = ~$0.124/hr (40% off on-demand $0.192/hr). Saves ~$112/mo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Set CloudWatch EKS log retention to 30 days</t>
+        </is>
+      </c>
+      <c r="C77" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>EKS cluster logs at 2.98GB with no retention. Set 30-day retention. aws logs put-retention-policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Delete orphaned KMS key</t>
+        </is>
+      </c>
+      <c r="C78" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>Key d514cb7e (alias removed). Schedule deletion to save $1/mo. Needs kms:ScheduleKeyDeletion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Delete orphaned CloudWatch log group</t>
+        </is>
+      </c>
+      <c r="C79" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>/aws/eks/le-shared-eks/cluster (173MB). Needs logs:DeleteLogGroup permission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Migrate gp2 → gp3 EBS volumes</t>
+        </is>
+      </c>
+      <c r="C80" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>54GB on gp2 ($0.114/GB) → gp3 ($0.0912/GB). ~15% savings on those volumes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Verify NAT Gateway is needed</t>
+        </is>
+      </c>
+      <c r="C81" s="12" t="n">
+        <v>18.76</v>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>NAT GW costs $18.76/mo but private subnets may not need egress. Delete if unused.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Delete finspot-cloud VPC + EFS</t>
+        </is>
+      </c>
+      <c r="C82" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>Orphaned VPC with EFS mount. Needs EFS permissions to clean up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="13" t="inlineStr"/>
+      <c r="B83" s="13" t="inlineStr">
+        <is>
+          <t>TOTAL POTENTIAL SAVINGS</t>
+        </is>
+      </c>
+      <c r="C83" s="14" t="n">
+        <v>504.76</v>
+      </c>
+      <c r="D83" s="13" t="inlineStr"/>
+      <c r="E83" s="13" t="inlineStr"/>
+      <c r="F83" s="13" t="inlineStr">
+        <is>
+          <t>Up to $504/mo = ~46% reduction</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A73:F73"/>
+    <mergeCell ref="A54:F54"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update CLAUDE.md and tracker for 2026-03-30 optimizations
- EKS control plane upgraded: v1.31 → v1.32 → v1.33 → v1.34
- CloudWatch logging disabled (not required)
- le-jenkins-ng node group deleted; merged into le-mgmt-tools-ng-v2
- le-mgmt-tools-ng-v2 scaled to 2 nodes (all workloads on single group)
- Excel tracker: resource IDs, cost projections, and savings summary updated
- Applied savings: ~$549/mo (EKS extended support + Jenkins node + CW logs)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LinkedEye_AWS_Resource_Tracker.xlsx
+++ b/LinkedEye_AWS_Resource_Tracker.xlsx
@@ -24,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +47,9 @@
     <font>
       <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="8">
@@ -139,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -176,6 +179,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1150,7 +1154,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>K8s v1.31, Platform eks.52</t>
+          <t>K8s v1.34 (control plane), logging disabled</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -1160,14 +1164,14 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Created 2026-03-12</t>
+          <t>Upgraded 2026-03-30: 1.31→1.32→1.33→1.34</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Node Group</t>
+          <t>Node Group (deleted)</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -1182,17 +1186,17 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>m5.xlarge, 50GB disk, AL2, 1/1/1 (min/desired/max)</t>
+          <t>m5.xlarge, AL2 — DELETED 2026-03-30</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Deleted</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Public subnet AZ1a</t>
+          <t>Merged into le-mgmt-tools-ng-v2</t>
         </is>
       </c>
     </row>
@@ -1209,12 +1213,12 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>i-08a738a53ecf2259d</t>
+          <t>eks-le-mgmt-tools-ng-v2-2ece838f-be29-bd78-d854-fa41dd941cd7</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>m5.xlarge, 100GB disk, AL2, 1/1/2 (min/desired/max)</t>
+          <t>2x m5.xlarge, AL2, 2/2/2 (min/desired/max) — nodes at v1.31</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -1224,7 +1228,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Public subnet AZ1a</t>
+          <t>Labels: role=mgmt-tools, jenkins=true. Node upgrade to v1.34 needs AL2023 AMI.</t>
         </is>
       </c>
     </row>
@@ -2254,17 +2258,17 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>EKS control plane logs (2.98 GB)</t>
+          <t>EKS control plane logs — DISABLED 2026-03-30</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Disabled</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>No retention set</t>
+          <t>Logging disabled to reduce CW costs</t>
         </is>
       </c>
     </row>
@@ -5753,7 +5757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F83"/>
+  <dimension ref="A1:F88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -6299,11 +6303,11 @@
           <t>DAILY SPEND TREND — March 2026</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="8" t="n"/>
+      <c r="E22" s="8" t="n"/>
+      <c r="F22" s="9" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
@@ -6835,11 +6839,11 @@
           <t>MONTHLY COST PROJECTION</t>
         </is>
       </c>
-      <c r="B54" s="3" t="n"/>
-      <c r="C54" s="3" t="n"/>
-      <c r="D54" s="3" t="n"/>
-      <c r="E54" s="3" t="n"/>
-      <c r="F54" s="3" t="n"/>
+      <c r="B54" s="8" t="n"/>
+      <c r="C54" s="8" t="n"/>
+      <c r="D54" s="8" t="n"/>
+      <c r="E54" s="8" t="n"/>
+      <c r="F54" s="9" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="15" t="inlineStr">
@@ -7155,11 +7159,11 @@
           <t>COST OPTIMIZATION RECOMMENDATIONS</t>
         </is>
       </c>
-      <c r="B73" s="3" t="n"/>
-      <c r="C73" s="3" t="n"/>
-      <c r="D73" s="3" t="n"/>
-      <c r="E73" s="3" t="n"/>
-      <c r="F73" s="3" t="n"/>
+      <c r="B73" s="8" t="n"/>
+      <c r="C73" s="8" t="n"/>
+      <c r="D73" s="8" t="n"/>
+      <c r="E73" s="8" t="n"/>
+      <c r="F73" s="9" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="15" t="inlineStr">
@@ -7199,7 +7203,7 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Upgrade EKS to v1.32+ (exit extended support)</t>
+          <t>Upgrade EKS v1.31→v1.34 (exit extended support) ✓ DONE 2026-03-30</t>
         </is>
       </c>
       <c r="C75" s="12" t="n">
@@ -7227,11 +7231,11 @@
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Reserved Instances for m5.xlarge nodes</t>
+          <t>Delete le-jenkins-ng, consolidate into le-mgmt-tools-ng-v2 ✓ DONE 2026-03-30</t>
         </is>
       </c>
       <c r="C76" s="12" t="n">
-        <v>112</v>
+        <v>177</v>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
@@ -7255,11 +7259,11 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Set CloudWatch EKS log retention to 30 days</t>
+          <t>Disable EKS CloudWatch logging (not required) ✓ DONE 2026-03-30</t>
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
@@ -7283,7 +7287,7 @@
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Delete orphaned KMS key</t>
+          <t>Delete orphaned KMS key d514cb7e (needs permission)</t>
         </is>
       </c>
       <c r="C78" s="12" t="n">
@@ -7311,7 +7315,7 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Delete orphaned CloudWatch log group</t>
+          <t>Delete orphaned CW log group /aws/eks/le-shared-eks (needs permission)</t>
         </is>
       </c>
       <c r="C79" s="12" t="n">
@@ -7367,7 +7371,7 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Verify NAT Gateway is needed</t>
+          <t>Verify/remove NAT Gateway if unused</t>
         </is>
       </c>
       <c r="C81" s="12" t="n">
@@ -7395,7 +7399,7 @@
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Delete finspot-cloud VPC + EFS</t>
+          <t>Delete finspot-cloud VPC + EFS (needs efs:DeleteMountTarget permission)</t>
         </is>
       </c>
       <c r="C82" s="12" t="n">
@@ -7421,11 +7425,11 @@
       <c r="A83" s="13" t="inlineStr"/>
       <c r="B83" s="13" t="inlineStr">
         <is>
-          <t>TOTAL POTENTIAL SAVINGS</t>
+          <t>TOTAL POTENTIAL SAVINGS (remaining: $22.76 after completed items)</t>
         </is>
       </c>
       <c r="C83" s="14" t="n">
-        <v>504.76</v>
+        <v>571.76</v>
       </c>
       <c r="D83" s="13" t="inlineStr"/>
       <c r="E83" s="13" t="inlineStr"/>
@@ -7433,6 +7437,63 @@
         <is>
           <t>Up to $504/mo = ~46% reduction</t>
         </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="16" t="inlineStr">
+        <is>
+          <t>APPLIED SAVINGS (2026-03-30)</t>
+        </is>
+      </c>
+      <c r="B84" s="16" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="C84" s="16" t="inlineStr">
+        <is>
+          <t>Monthly Saving (USD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>EKS v1.31 → v1.34 upgrade (extended support removed)</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>le-jenkins-ng node group deleted (2nd m5.xlarge)</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>EKS CloudWatch logging disabled</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="16" t="inlineStr">
+        <is>
+          <t>TOTAL APPLIED SAVINGS</t>
+        </is>
+      </c>
+      <c r="C88" s="16" t="n">
+        <v>549</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update cost details with actual AWS figures (2026-03-30)
- March actual: $874 (verified via Cost Explorer)
- April projected: ~$510 (daily rate ~$17/day, was $31/day)
- Applied savings: $372/mo (EKS extended support $365 + CW logs $7)
- Added Monthly Cost section to CLAUDE.md
- Excel: all service rows updated with real amounts and April projections

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LinkedEye_AWS_Resource_Tracker.xlsx
+++ b/LinkedEye_AWS_Resource_Tracker.xlsx
@@ -5757,7 +5757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:F89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -5823,7 +5823,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2x m5.xlarge (node groups) + m5.2xlarge + m5.4xlarge</t>
+          <t>m5.xlarge x853h + m5.4xlarge x97h + m5.2xlarge x174h</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -5833,7 +5833,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>m5.4xlarge terminated mid-month; consider Reserved Instances for steady-state nodes</t>
+          <t>April projected: $140 (2x m5.xlarge; jenkins-ng deleted)</t>
         </is>
       </c>
     </row>
@@ -5863,7 +5863,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Fixed $0.10/hr — no optimization possible</t>
+          <t>April projected: $73 (fixed $0.10/hr x 730hr)</t>
         </is>
       </c>
     </row>
@@ -5883,17 +5883,17 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>EKS v1.31 extended support surcharge</t>
+          <t>v1.31 extended support ELIMINATED (upgraded to v1.34 on 2026-03-30)</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>446 hours @ $0.50/hr</t>
+          <t>$0.50/hr x 446hr</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>UPGRADE to v1.32+ when available to exit extended support ($0.50/hr savings)</t>
+          <t>April projected: $0 — SAVING $365/mo</t>
         </is>
       </c>
     </row>
@@ -5923,7 +5923,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Scales with client count; currently 15 clients</t>
+          <t>April projected: $53 (same — 15 clients unchanged)</t>
         </is>
       </c>
     </row>
@@ -6063,7 +6063,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>VPC Flow Logs, EKS logs</t>
+          <t>VPC Flow Logs + EKS control plane logs (logging disabled 2026-03-30)</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -6073,7 +6073,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Set retention on EKS logs (currently unlimited — 2.98 GB growing)</t>
+          <t>April projected: $3 — SAVING $7/mo</t>
         </is>
       </c>
     </row>
@@ -6286,16 +6286,45 @@
         </is>
       </c>
       <c r="B20" s="14" t="n">
-        <v>873.75</v>
+        <v>874</v>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="D20" s="13" t="inlineStr"/>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>Verified via AWS Cost Explorer 2026-03-30</t>
+        </is>
+      </c>
       <c r="E20" s="13" t="inlineStr"/>
       <c r="F20" s="13" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TOTAL (April 2026 projected after optimizations)</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>510</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Daily rate: ~$17/day x 30 days</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Saving: $364/mo vs March</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>EKS extended support eliminated + logging disabled</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -7442,7 +7471,7 @@
     <row r="84">
       <c r="A84" s="16" t="inlineStr">
         <is>
-          <t>APPLIED SAVINGS (2026-03-30)</t>
+          <t>OPTIMIZATION SUMMARY — Applied 2026-03-30</t>
         </is>
       </c>
       <c r="B84" s="16" t="inlineStr">
@@ -7457,44 +7486,92 @@
       </c>
     </row>
     <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>EKS v1.31 → v1.34 upgrade (extended support removed)</t>
-        </is>
-      </c>
-      <c r="C85" t="n">
+          <t>Action Taken</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Monthly Saving (USD)</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>1</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>EKS v1.31 to v1.34 upgrade (extended support $0.50/hr removed)</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
         <v>365</v>
       </c>
-    </row>
-    <row r="86">
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>le-jenkins-ng node group deleted (2nd m5.xlarge)</t>
-        </is>
-      </c>
-      <c r="C86" t="n">
-        <v>177</v>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Done 2026-03-30</t>
+        </is>
       </c>
     </row>
     <row r="87">
+      <c r="A87" t="n">
+        <v>2</v>
+      </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>EKS CloudWatch logging disabled</t>
+          <t>EKS CloudWatch control plane logging disabled</t>
         </is>
       </c>
       <c r="C87" t="n">
         <v>7</v>
       </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Done 2026-03-30</t>
+        </is>
+      </c>
     </row>
     <row r="88">
+      <c r="A88" t="n">
+        <v>3</v>
+      </c>
       <c r="B88" s="16" t="inlineStr">
         <is>
+          <t>le-jenkins-ng deleted; workloads merged into le-mgmt-tools-ng-v2 (2 nodes)</t>
+        </is>
+      </c>
+      <c r="C88" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Done 2026-03-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr"/>
+      <c r="B89" t="inlineStr">
+        <is>
           <t>TOTAL APPLIED SAVINGS</t>
         </is>
       </c>
-      <c r="C88" s="16" t="n">
-        <v>549</v>
-      </c>
+      <c r="C89" t="n">
+        <v>372</v>
+      </c>
+      <c r="D89" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Upgrade node group to AL2023 with K8s v1.34
- Created le-mgmt-tools-ng-v3 (AL2023, K8s v1.34, 2x m5.xlarge)
- Drained and deleted le-mgmt-tools-ng-v2 (AL2, K8s v1.31)
- All workloads migrated to new nodes successfully
- Fixed IMDS hop limit (1→2) for EBS CSI volume attachment
- Jenkins nodeSelector fixed: role=jenkins → jenkins=true
- Deployed Prometheus + Grafana monitoring stack to le-monitoring
- Full stack: Jenkins, ArgoCD, Harbor, Keycloak, Vault, MinIO, PostgreSQL, Prometheus/Grafana all running

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LinkedEye_AWS_Resource_Tracker.xlsx
+++ b/LinkedEye_AWS_Resource_Tracker.xlsx
@@ -1154,7 +1154,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>K8s v1.34 (control plane), logging disabled</t>
+          <t>K8s v1.34, AL2023 nodes, logging disabled</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Upgraded 2026-03-30: 1.31→1.32→1.33→1.34</t>
+          <t>Upgraded 2026-03-30/31: v1.31→v1.34, AL2→AL2023</t>
         </is>
       </c>
     </row>
@@ -1208,17 +1208,17 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>le-mgmt-tools-ng-v2</t>
+          <t>le-mgmt-tools-ng-v3</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>eks-le-mgmt-tools-ng-v2-2ece838f-be29-bd78-d854-fa41dd941cd7</t>
+          <t>2x m5.xlarge (AL2023, K8s v1.34)</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2x m5.xlarge, AL2, 2/2/2 (min/desired/max) — nodes at v1.31</t>
+          <t>2x m5.xlarge, AL2023, 2/2/2 (min/desired/max)</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Labels: role=mgmt-tools, jenkins=true. Node upgrade to v1.34 needs AL2023 AMI.</t>
+          <t>Labels: role=mgmt-tools, jenkins=true. Replaced le-mgmt-tools-ng-v2 (AL2).</t>
         </is>
       </c>
     </row>
@@ -4250,7 +4250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -4554,6 +4554,33 @@
       <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Claude Code</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Node Group</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>le-mgmt-tools-ng-v2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>AL2, K8s v1.31</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Replaced by le-mgmt-tools-ng-v3 (AL2023, K8s v1.34)</t>
         </is>
       </c>
     </row>
@@ -7562,7 +7589,6 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr"/>
       <c r="B89" t="inlineStr">
         <is>
           <t>TOTAL APPLIED SAVINGS</t>
@@ -7571,7 +7597,6 @@
       <c r="C89" t="n">
         <v>372</v>
       </c>
-      <c r="D89" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Update ALB routing and tool URLs in tracker
- All target groups registered with new v1.34 node instances
- Added le-itsm.api.finspot.in ALB rule (priority 8)
- Tools & Services sheet: correct FQDNs, NodePorts, running status
- Node group updated to le-mgmt-tools-ng-v3 (AL2023)
- All tools healthy: Jenkins, ArgoCD, Harbor, Keycloak, Vault, MinIO, Prometheus/Grafana

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LinkedEye_AWS_Resource_Tracker.xlsx
+++ b/LinkedEye_AWS_Resource_Tracker.xlsx
@@ -3692,17 +3692,17 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>le-jenkins-ng (m5.xlarge)</t>
+          <t>le-mgmt-tools-ng-v3 (2x m5.xlarge, AL2023)</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>8080</t>
+          <t>30080</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>jenkins.finspot.in</t>
+          <t>le-jenkins.finspot.in</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -3712,12 +3712,12 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>CI/CD pipeline</t>
+          <t>NodePort 30080, nodeSelector: jenkins=true</t>
         </is>
       </c>
     </row>
@@ -3729,17 +3729,17 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>le-mgmt-tools-ng-v2 (m5.xlarge)</t>
+          <t>le-mgmt-tools-ng-v3</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>8082</t>
+          <t>30082</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>argocd.finspot.in</t>
+          <t>le-argocd.finspot.in</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -3749,12 +3749,12 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>GitOps deployment</t>
+          <t>NodePort 30082</t>
         </is>
       </c>
     </row>
@@ -3766,17 +3766,17 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>le-mgmt-tools-ng-v2</t>
+          <t>le-mgmt-tools-ng-v3</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>8083</t>
+          <t>30083</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>harbor.finspot.in</t>
+          <t>le-harbor.finspot.in</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -3786,12 +3786,12 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Container registry</t>
+          <t>Portal NodePort 30083, Registry 30500</t>
         </is>
       </c>
     </row>
@@ -3803,17 +3803,17 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>le-mgmt-tools-ng-v2</t>
+          <t>le-mgmt-tools-ng-v3</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>8081</t>
+          <t>30081</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>keycloak.finspot.in</t>
+          <t>le-keycloak.finspot.in</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -3823,12 +3823,12 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>SSO / Identity</t>
+          <t>NodePort 30081</t>
         </is>
       </c>
     </row>
@@ -3840,17 +3840,17 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>le-mgmt-tools-ng-v2</t>
+          <t>le-mgmt-tools-ng-v3</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>8200</t>
+          <t>30200</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>vault.finspot.in</t>
+          <t>le-vault.finspot.in</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -3860,12 +3860,12 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Secrets management</t>
+          <t>NodePort 30200</t>
         </is>
       </c>
     </row>
@@ -3877,7 +3877,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>le-mgmt-tools-ng-v2</t>
+          <t>le-mgmt-tools-ng-v3</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>fs-le-*.finspot.in</t>
+          <t>le-itsm.finspot.in</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -3897,7 +3897,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Configured</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -3909,12 +3909,12 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Client ITSM</t>
+          <t>ITSM API</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>le-mgmt-tools-ng-v2</t>
+          <t>le-mgmt-tools-ng-v3</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -3924,118 +3924,118 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>fs-le-{client}.finspot.in</t>
+          <t>le-itsm.api.finspot.in</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>linkedeye-tg-client-itsm</t>
+          <t>linkedeye-tg-itsm</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Script Ready</t>
+          <t>Configured</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>15 client FQDNs</t>
+          <t>ALB rule priority 8 (added 2026-03-31)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>MinIO</t>
+          <t>Client ITSM</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>le-mgmt-tools-ng-v2</t>
+          <t>Hybrid nodes (on-prem per client)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>30901</t>
+          <t>80</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>18 client FQDNs (priorities 10-27)</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>linkedeye-tg-minio</t>
+          <t>linkedeye-tg-client-itsm</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Configured</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Object storage</t>
+          <t>15 prod + 3 non-prod client FQDNs</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Prometheus</t>
+          <t>MinIO</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>EKS (kube-prometheus-stack)</t>
+          <t>le-mgmt-tools-ng-v3</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>9090</t>
+          <t>31114</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>le-minio.finspot.in (internal)</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>linkedeye-tg-minio</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>12-enterprise/11</t>
+          <t>Console NodePort 31114, API 30147</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Grafana</t>
+          <t>Prometheus</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>EKS (kube-prometheus-stack)</t>
+          <t>le-mgmt-tools-ng-v3 (le-monitoring ns)</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>3000</t>
+          <t>9090</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>grafana.finspot.in</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -4045,29 +4045,29 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>12-enterprise/11</t>
+          <t>kube-prometheus-stack, 50Gi storage, 30d retention</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Alertmanager</t>
+          <t>Grafana</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>EKS (kube-prometheus-stack)</t>
+          <t>le-mgmt-tools-ng-v3 (le-monitoring ns)</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>9093</t>
+          <t>30090</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -4082,29 +4082,29 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>→ StackStorm st2api:9101</t>
+          <t>NodePort 30090, admin/LinkedEye@Grafana2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Velero</t>
+          <t>Alertmanager</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>EKS</t>
+          <t>le-mgmt-tools-ng-v3 (le-monitoring ns)</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9093</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -4119,29 +4119,29 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>S3 backup bucket created</t>
+          <t>Webhooks → StackStorm st2api:9101</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>External Secrets</t>
+          <t>PostgreSQL</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>EKS</t>
+          <t>le-mgmt-tools-ng-v3 (le-postgres ns)</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5432</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -4156,24 +4156,24 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Vault → K8s sync</t>
+          <t>ClusterIP 172.20.67.14, used by Jenkins/Harbor/Keycloak</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>GuardDuty Agent</t>
+          <t>Velero</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>EKS Addon</t>
+          <t>EKS</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -4198,19 +4198,19 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>v1.12.1</t>
+          <t>S3 bucket: linkedeye-velero-backups-654697417727</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Container Insights</t>
+          <t>GuardDuty Agent</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>EKS</t>
+          <t>EKS Addon</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -4230,12 +4230,12 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>CloudWatch monitoring</t>
+          <t>v1.12.1 addon</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update docs: hybrid nodes, monitoring, IAM, CoreDNS fixes
- 2 hybrid on-prem nodes registered (192.168.100.72, 172.16.0.62)
- Prometheus/Grafana/Alertmanager deployed to le-monitoring
- CoreDNS fixed: hostNetwork=true, nodeSelector=mgmt-tools
- IAM policy LinkedEye-DevOps-Extra added (SSM, ECR, EC2-Connect, EFS, KMS)
- ALB: 8 tool + 18 client rules, sticky sessions enabled
- Jenkins: admin user reset, CSRF proxy fix, plugin downloads working
- ArgoCD: admin password reset
- MinIO: MINIO_SERVER_URL fixed to internal service
- All tool logins verified working

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LinkedEye_AWS_Resource_Tracker.xlsx
+++ b/LinkedEye_AWS_Resource_Tracker.xlsx
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1380,27 +1380,27 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>On-prem workers (15 clients)</t>
+          <t>mi-071e737d121051583, mi-0e0c4253be3fb4d14</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>192.168.100.72, 172.16.0.62</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>SSM Hybrid Activation, public API</t>
+          <t>2 on-prem Ubuntu 22.04 nodes (SSM registered)</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>No VPN needed</t>
+          <t>Registered via SSM Hybrid Activation 8edaa66d</t>
         </is>
       </c>
     </row>
@@ -2009,44 +2009,48 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>IAM Policy</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>LinkedEye-DevOps-Extra</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>arn:aws:iam::654697417727:policy/LinkedEye-DevOps-Extra</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>SSM, ECR, EC2-Connect, EFS, KMS delete, CW Logs delete</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Attached to rajkumar.madhu@finspot.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>SECURITY &amp; ENCRYPTION</t>
         </is>
       </c>
-      <c r="B52" s="8" t="n"/>
-      <c r="C52" s="8" t="n"/>
-      <c r="D52" s="8" t="n"/>
-      <c r="E52" s="8" t="n"/>
-      <c r="F52" s="9" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>KMS Key</t>
-        </is>
-      </c>
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>linkedeye-kms-eks</t>
-        </is>
-      </c>
-      <c r="C53" s="4" t="inlineStr">
-        <is>
-          <t>79f25c77-3399-457e-9981-61ab6a59440f</t>
-        </is>
-      </c>
-      <c r="D53" s="4" t="inlineStr">
-        <is>
-          <t>EKS secrets encryption</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="inlineStr"/>
+      <c r="B53" s="8" t="n"/>
+      <c r="C53" s="8" t="n"/>
+      <c r="D53" s="8" t="n"/>
+      <c r="E53" s="8" t="n"/>
+      <c r="F53" s="9" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -2056,17 +2060,17 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>linkedeye-kms-vault</t>
+          <t>linkedeye-kms-eks</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>6e42d4e7-7d23-48c3-9956-47e3e3ec79f0</t>
+          <t>79f25c77-3399-457e-9981-61ab6a59440f</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Vault auto-unseal</t>
+          <t>EKS secrets encryption</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -2084,17 +2088,17 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>linkedeye-kms-ebs</t>
+          <t>linkedeye-kms-vault</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>c58c1e22-a9a7-48f3-a5f1-f50d67c6695e</t>
+          <t>6e42d4e7-7d23-48c3-9956-47e3e3ec79f0</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>EBS volume encryption</t>
+          <t>Vault auto-unseal</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -2107,22 +2111,22 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>WAF</t>
+          <t>KMS Key</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>linkedeye-waf</t>
+          <t>linkedeye-kms-ebs</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>c125267b-4e92-4c24-8a03-88eddcdc3be7</t>
+          <t>c58c1e22-a9a7-48f3-a5f1-f50d67c6695e</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>4 rules: CommonRuleSet, KnownBadInputs, SQLi, RateLimit</t>
+          <t>EBS volume encryption</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -2130,83 +2134,79 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>Attached to ALB</t>
-        </is>
-      </c>
+      <c r="F56" s="4" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
+          <t>WAF</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>linkedeye-waf</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>c125267b-4e92-4c24-8a03-88eddcdc3be7</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>4 rules: CommonRuleSet, KnownBadInputs, SQLi, RateLimit</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>Attached to ALB</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
           <t>GuardDuty</t>
         </is>
       </c>
-      <c r="B57" s="4" t="inlineStr">
+      <c r="B58" s="4" t="inlineStr">
         <is>
           <t>Detector</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
+      <c r="C58" s="4" t="inlineStr">
         <is>
           <t>fa47792e40684b45bfa76c1b4a1a48a4</t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr">
+      <c r="D58" s="4" t="inlineStr">
         <is>
           <t>Threat detection</t>
         </is>
       </c>
-      <c r="E57" s="5" t="inlineStr">
+      <c r="E58" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="F57" s="4" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="F58" s="4" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>STORAGE &amp; LOGGING</t>
         </is>
       </c>
-      <c r="B58" s="8" t="n"/>
-      <c r="C58" s="8" t="n"/>
-      <c r="D58" s="8" t="n"/>
-      <c r="E58" s="8" t="n"/>
-      <c r="F58" s="9" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>S3 Bucket</t>
-        </is>
-      </c>
-      <c r="B59" s="4" t="inlineStr">
-        <is>
-          <t>linkedeye-velero-backups-654697417727</t>
-        </is>
-      </c>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t>Velero cluster backups</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F59" s="4" t="inlineStr">
-        <is>
-          <t>Created 2026-03-10</t>
-        </is>
-      </c>
+      <c r="B59" s="8" t="n"/>
+      <c r="C59" s="8" t="n"/>
+      <c r="D59" s="8" t="n"/>
+      <c r="E59" s="8" t="n"/>
+      <c r="F59" s="9" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>linkedeye-audit-logs-654697417727</t>
+          <t>linkedeye-velero-backups-654697417727</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>CloudTrail audit logs</t>
+          <t>Velero cluster backups</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -2243,12 +2243,12 @@
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>CloudWatch Logs</t>
+          <t>S3 Bucket</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>/aws/eks/linkedeye-finspot-k8s-cluster/cluster</t>
+          <t>linkedeye-audit-logs-654697417727</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -2258,17 +2258,17 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>EKS control plane logs — DISABLED 2026-03-30</t>
+          <t>CloudTrail audit logs</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>Disabled</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>Logging disabled to reduce CW costs</t>
+          <t>Created 2026-03-10</t>
         </is>
       </c>
     </row>
@@ -2280,129 +2280,161 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
+          <t>/aws/eks/linkedeye-finspot-k8s-cluster/cluster</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>EKS control plane logs — DISABLED 2026-03-30</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>Logging disabled to reduce CW costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>CloudWatch Logs</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
           <t>/aws/vpc/flowlogs/linkedeye</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D62" s="4" t="inlineStr">
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
         <is>
           <t>VPC flow logs (23 MB, 90-day retention)</t>
         </is>
       </c>
-      <c r="E62" s="5" t="inlineStr">
+      <c r="E63" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="F62" s="4" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+      <c r="F63" s="4" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>ORPHANED RESOURCES (needs cleanup)</t>
         </is>
       </c>
-      <c r="B63" s="8" t="n"/>
-      <c r="C63" s="8" t="n"/>
-      <c r="D63" s="8" t="n"/>
-      <c r="E63" s="8" t="n"/>
-      <c r="F63" s="9" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="4" t="inlineStr">
-        <is>
-          <t>CloudWatch Logs</t>
-        </is>
-      </c>
-      <c r="B64" s="4" t="inlineStr">
-        <is>
-          <t>/aws/eks/le-shared-eks/cluster</t>
-        </is>
-      </c>
-      <c r="C64" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D64" s="4" t="inlineStr">
-        <is>
-          <t>173 MB from deleted cluster</t>
-        </is>
-      </c>
-      <c r="E64" s="7" t="inlineStr">
-        <is>
-          <t>Orphan — Delete</t>
-        </is>
-      </c>
-      <c r="F64" s="4" t="inlineStr">
-        <is>
-          <t>Need logs:DeleteLogGroup permission</t>
-        </is>
-      </c>
+      <c r="B64" s="8" t="n"/>
+      <c r="C64" s="8" t="n"/>
+      <c r="D64" s="8" t="n"/>
+      <c r="E64" s="8" t="n"/>
+      <c r="F64" s="9" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>KMS Key</t>
+          <t>CloudWatch Logs</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>(alias removed, unnamed)</t>
+          <t>/aws/eks/le-shared-eks/cluster</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>d514cb7e-6ce0-4d17-a42d-a0311ded34d0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Unused EKS secrets key</t>
+          <t>173 MB from deleted cluster</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>Orphan — Disable/Delete</t>
+          <t>Orphan — Delete</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>Need kms:ScheduleKeyDeletion</t>
+          <t>Need logs:DeleteLogGroup permission</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
+          <t>KMS Key</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>(alias removed, unnamed)</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>d514cb7e-6ce0-4d17-a42d-a0311ded34d0</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>Unused EKS secrets key</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>Orphan — Disable/Delete</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>Need kms:ScheduleKeyDeletion</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
           <t>VPC</t>
         </is>
       </c>
-      <c r="B66" s="4" t="inlineStr">
+      <c r="B67" s="4" t="inlineStr">
         <is>
           <t>finspot-cloud</t>
         </is>
       </c>
-      <c r="C66" s="4" t="inlineStr">
+      <c r="C67" s="4" t="inlineStr">
         <is>
           <t>vpc-0bd83076448a26cec</t>
         </is>
       </c>
-      <c r="D66" s="4" t="inlineStr">
+      <c r="D67" s="4" t="inlineStr">
         <is>
           <t>11.0.0.0/24, empty except EFS mount</t>
         </is>
       </c>
-      <c r="E66" s="7" t="inlineStr">
+      <c r="E67" s="7" t="inlineStr">
         <is>
           <t>Orphan — Delete</t>
         </is>
       </c>
-      <c r="F66" s="4" t="inlineStr">
+      <c r="F67" s="4" t="inlineStr">
         <is>
           <t>Need efs:DeleteMountTarget first</t>
         </is>

</xml_diff>